<commit_message>
Planilha financeira de desenvolvimento
Com link
</commit_message>
<xml_diff>
--- a/docs/Planilha financeira de desenvolvimento.xlsx
+++ b/docs/Planilha financeira de desenvolvimento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guilh\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F435944-66A5-43CA-B7F5-F38BD103BFA2}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E7F8017-A38C-434B-B2DC-B20E81F6F6A0}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="79">
   <si>
     <t>Receita</t>
   </si>
@@ -298,7 +298,10 @@
     <t>(R$71,42/Colaborador)</t>
   </si>
   <si>
-    <t>Link do documento</t>
+    <t>https://github.com/ryatsuga/cosmos/blob/master/docs/Planilha%20financeira%20de%20desenvolvimento.xlsx</t>
+  </si>
+  <si>
+    <t>Link do documento:</t>
   </si>
 </sst>
 </file>
@@ -308,7 +311,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="34">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -494,6 +497,12 @@
       <color indexed="9"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="12">
@@ -747,11 +756,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -835,33 +845,80 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="49" fontId="25" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="27" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="23" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -890,98 +947,55 @@
     <xf numFmtId="0" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="28" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="27" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="23" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="9" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
@@ -1803,10 +1817,10 @@
       <c r="P2" s="49"/>
     </row>
     <row r="3" spans="1:17" s="5" customFormat="1" ht="21" customHeight="1">
-      <c r="A3" s="57"/>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
+      <c r="A3" s="106"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="106"/>
+      <c r="D3" s="106"/>
       <c r="E3" s="15" t="s">
         <v>9</v>
       </c>
@@ -1832,12 +1846,12 @@
       <c r="Q3" s="7"/>
     </row>
     <row r="4" spans="1:17" s="6" customFormat="1" ht="15" customHeight="1">
-      <c r="A4" s="109" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="81"/>
-      <c r="C4" s="81"/>
-      <c r="D4" s="81"/>
+      <c r="A4" s="108" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="109"/>
+      <c r="C4" s="109"/>
+      <c r="D4" s="109"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
       <c r="G4" s="16"/>
@@ -1853,10 +1867,12 @@
       <c r="Q4" s="8"/>
     </row>
     <row r="5" spans="1:17" s="6" customFormat="1" ht="15" customHeight="1">
-      <c r="A5" s="81"/>
-      <c r="B5" s="81"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="81"/>
+      <c r="A5" s="110" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="109"/>
+      <c r="C5" s="109"/>
+      <c r="D5" s="109"/>
       <c r="E5" s="17" t="s">
         <v>3</v>
       </c>
@@ -1882,27 +1898,27 @@
       <c r="Q5" s="8"/>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1">
-      <c r="A6" s="82" t="s">
+      <c r="A6" s="83" t="s">
         <v>63</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="90" t="s">
+      <c r="B6" s="107"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="66" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="100">
+      <c r="E6" s="72">
         <v>7973.65</v>
       </c>
-      <c r="F6" s="101">
+      <c r="F6" s="73">
         <v>4026.35</v>
       </c>
-      <c r="G6" s="102" t="s">
+      <c r="G6" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H6" s="103" t="s">
+      <c r="H6" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I6" s="102" t="s">
+      <c r="I6" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J6" s="13"/>
@@ -1915,25 +1931,25 @@
       <c r="Q6" s="9"/>
     </row>
     <row r="7" spans="1:17" ht="15" customHeight="1">
-      <c r="A7" s="58"/>
-      <c r="B7" s="58"/>
-      <c r="C7" s="58"/>
-      <c r="D7" s="90" t="s">
+      <c r="A7" s="107"/>
+      <c r="B7" s="107"/>
+      <c r="C7" s="107"/>
+      <c r="D7" s="66" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="100">
+      <c r="E7" s="72">
         <v>0</v>
       </c>
-      <c r="F7" s="103" t="s">
+      <c r="F7" s="75" t="s">
         <v>69</v>
       </c>
-      <c r="G7" s="102" t="s">
+      <c r="G7" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H7" s="103" t="s">
+      <c r="H7" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I7" s="102" t="s">
+      <c r="I7" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J7" s="13"/>
@@ -1946,15 +1962,15 @@
       <c r="Q7" s="9"/>
     </row>
     <row r="8" spans="1:17" ht="3" customHeight="1">
-      <c r="A8" s="58"/>
-      <c r="B8" s="58"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="83"/>
-      <c r="E8" s="84"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="84"/>
-      <c r="H8" s="84"/>
-      <c r="I8" s="84"/>
+      <c r="A8" s="107"/>
+      <c r="B8" s="107"/>
+      <c r="C8" s="107"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="61"/>
+      <c r="I8" s="61"/>
       <c r="J8" s="13"/>
       <c r="K8" s="9"/>
       <c r="L8" s="9"/>
@@ -1965,29 +1981,29 @@
       <c r="Q8" s="9"/>
     </row>
     <row r="9" spans="1:17" ht="15" customHeight="1">
-      <c r="A9" s="58"/>
-      <c r="B9" s="58"/>
-      <c r="C9" s="58"/>
-      <c r="D9" s="85" t="s">
+      <c r="A9" s="107"/>
+      <c r="B9" s="107"/>
+      <c r="C9" s="107"/>
+      <c r="D9" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="86">
+      <c r="E9" s="63">
         <f>SUM(E6:E7)</f>
         <v>7973.65</v>
       </c>
-      <c r="F9" s="86">
+      <c r="F9" s="63">
         <f>SUM(F6:F7)</f>
         <v>4026.35</v>
       </c>
-      <c r="G9" s="86">
+      <c r="G9" s="63">
         <f>SUM(G6:G7)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="86">
+      <c r="H9" s="63">
         <f>SUM(H6:H7)</f>
         <v>0</v>
       </c>
-      <c r="I9" s="86">
+      <c r="I9" s="63">
         <f>SUM(I6:I7)</f>
         <v>0</v>
       </c>
@@ -2001,15 +2017,15 @@
       <c r="Q9" s="9"/>
     </row>
     <row r="10" spans="1:17" ht="15" customHeight="1">
-      <c r="A10" s="82" t="s">
+      <c r="A10" s="83" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="82"/>
-      <c r="C10" s="89"/>
-      <c r="D10" s="87" t="s">
+      <c r="B10" s="83"/>
+      <c r="C10" s="84"/>
+      <c r="D10" s="64" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="88">
+      <c r="E10" s="65">
         <v>12000</v>
       </c>
       <c r="F10" s="13"/>
@@ -2025,13 +2041,13 @@
       <c r="P10" s="3"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1">
-      <c r="A11" s="82"/>
-      <c r="B11" s="82"/>
-      <c r="C11" s="89"/>
-      <c r="D11" s="87" t="s">
+      <c r="A11" s="83"/>
+      <c r="B11" s="83"/>
+      <c r="C11" s="84"/>
+      <c r="D11" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="88">
+      <c r="E11" s="65">
         <v>100000</v>
       </c>
       <c r="F11" s="13"/>
@@ -2047,13 +2063,13 @@
       <c r="P11" s="3"/>
     </row>
     <row r="12" spans="1:17" ht="15" customHeight="1">
-      <c r="A12" s="82"/>
-      <c r="B12" s="82"/>
-      <c r="C12" s="89"/>
-      <c r="D12" s="92" t="s">
+      <c r="A12" s="83"/>
+      <c r="B12" s="83"/>
+      <c r="C12" s="84"/>
+      <c r="D12" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="93">
+      <c r="E12" s="68">
         <v>112000</v>
       </c>
       <c r="F12" s="13"/>
@@ -2069,11 +2085,11 @@
       <c r="P12" s="3"/>
     </row>
     <row r="13" spans="1:17" s="6" customFormat="1" ht="15.95" customHeight="1">
-      <c r="A13" s="55" t="s">
+      <c r="A13" s="104" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="55"/>
-      <c r="C13" s="55"/>
+      <c r="B13" s="104"/>
+      <c r="C13" s="104"/>
       <c r="D13" s="22"/>
       <c r="E13" s="23"/>
       <c r="F13" s="23"/>
@@ -2090,9 +2106,9 @@
       <c r="Q13" s="8"/>
     </row>
     <row r="14" spans="1:17" ht="17.100000000000001" customHeight="1">
-      <c r="A14" s="55"/>
-      <c r="B14" s="55"/>
-      <c r="C14" s="55"/>
+      <c r="A14" s="104"/>
+      <c r="B14" s="104"/>
+      <c r="C14" s="104"/>
       <c r="D14" s="25"/>
       <c r="E14" s="26"/>
       <c r="F14" s="26"/>
@@ -2109,9 +2125,9 @@
       <c r="Q14" s="9"/>
     </row>
     <row r="15" spans="1:17" s="6" customFormat="1" ht="15.95" customHeight="1">
-      <c r="A15" s="55"/>
-      <c r="B15" s="55"/>
-      <c r="C15" s="55"/>
+      <c r="A15" s="104"/>
+      <c r="B15" s="104"/>
+      <c r="C15" s="104"/>
       <c r="D15" s="22"/>
       <c r="E15" s="17"/>
       <c r="F15" s="17"/>
@@ -2128,27 +2144,27 @@
       <c r="Q15" s="8"/>
     </row>
     <row r="16" spans="1:17" ht="15" customHeight="1">
-      <c r="A16" s="94" t="s">
+      <c r="A16" s="103" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="94"/>
-      <c r="C16" s="94"/>
-      <c r="D16" s="90" t="s">
+      <c r="B16" s="103"/>
+      <c r="C16" s="103"/>
+      <c r="D16" s="66" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="100">
+      <c r="E16" s="72">
         <v>0</v>
       </c>
-      <c r="F16" s="101">
+      <c r="F16" s="73">
         <v>2855.35</v>
       </c>
-      <c r="G16" s="100">
+      <c r="G16" s="72">
         <v>5712.75</v>
       </c>
-      <c r="H16" s="101">
+      <c r="H16" s="73">
         <v>5712.75</v>
       </c>
-      <c r="I16" s="100">
+      <c r="I16" s="72">
         <v>5712.75</v>
       </c>
       <c r="J16" s="13"/>
@@ -2161,25 +2177,25 @@
       <c r="Q16" s="9"/>
     </row>
     <row r="17" spans="1:17">
-      <c r="A17" s="94"/>
-      <c r="B17" s="94"/>
-      <c r="C17" s="94"/>
+      <c r="A17" s="103"/>
+      <c r="B17" s="103"/>
+      <c r="C17" s="103"/>
       <c r="D17" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E17" s="100">
+      <c r="E17" s="72">
         <v>0</v>
       </c>
-      <c r="F17" s="101">
+      <c r="F17" s="73">
         <v>0</v>
       </c>
-      <c r="G17" s="102" t="s">
+      <c r="G17" s="74" t="s">
         <v>65</v>
       </c>
-      <c r="H17" s="103" t="s">
+      <c r="H17" s="75" t="s">
         <v>65</v>
       </c>
-      <c r="I17" s="102" t="s">
+      <c r="I17" s="74" t="s">
         <v>65</v>
       </c>
       <c r="J17" s="13"/>
@@ -2192,9 +2208,9 @@
       <c r="Q17" s="9"/>
     </row>
     <row r="18" spans="1:17" ht="3" customHeight="1">
-      <c r="A18" s="94"/>
-      <c r="B18" s="94"/>
-      <c r="C18" s="94"/>
+      <c r="A18" s="103"/>
+      <c r="B18" s="103"/>
+      <c r="C18" s="103"/>
       <c r="D18" s="19"/>
       <c r="E18" s="27"/>
       <c r="F18" s="27"/>
@@ -2211,9 +2227,9 @@
       <c r="Q18" s="9"/>
     </row>
     <row r="19" spans="1:17">
-      <c r="A19" s="94"/>
-      <c r="B19" s="94"/>
-      <c r="C19" s="94"/>
+      <c r="A19" s="103"/>
+      <c r="B19" s="103"/>
+      <c r="C19" s="103"/>
       <c r="D19" s="20" t="s">
         <v>15</v>
       </c>
@@ -2247,9 +2263,9 @@
       <c r="Q19" s="9"/>
     </row>
     <row r="20" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A20" s="94"/>
-      <c r="B20" s="94"/>
-      <c r="C20" s="94"/>
+      <c r="A20" s="103"/>
+      <c r="B20" s="103"/>
+      <c r="C20" s="103"/>
       <c r="D20" s="28"/>
       <c r="E20" s="26"/>
       <c r="F20" s="26"/>
@@ -2266,11 +2282,11 @@
       <c r="Q20" s="9"/>
     </row>
     <row r="21" spans="1:17">
-      <c r="A21" s="56" t="s">
+      <c r="A21" s="105" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="56"/>
-      <c r="C21" s="56"/>
+      <c r="B21" s="105"/>
+      <c r="C21" s="105"/>
       <c r="D21" s="30"/>
       <c r="E21" s="31"/>
       <c r="F21" s="31"/>
@@ -2287,9 +2303,9 @@
       <c r="Q21" s="9"/>
     </row>
     <row r="22" spans="1:17" ht="16.5">
-      <c r="A22" s="56"/>
-      <c r="B22" s="56"/>
-      <c r="C22" s="56"/>
+      <c r="A22" s="105"/>
+      <c r="B22" s="105"/>
+      <c r="C22" s="105"/>
       <c r="D22" s="24"/>
       <c r="E22" s="31"/>
       <c r="F22" s="31"/>
@@ -2307,10 +2323,10 @@
     </row>
     <row r="23" spans="1:17">
       <c r="A23" s="50"/>
-      <c r="B23" s="73" t="s">
+      <c r="B23" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="73"/>
+      <c r="C23" s="94"/>
       <c r="D23" s="54" t="s">
         <v>29</v>
       </c>
@@ -2319,7 +2335,7 @@
       <c r="G23" s="17"/>
       <c r="H23" s="17"/>
       <c r="I23" s="17"/>
-      <c r="J23" s="79" t="s">
+      <c r="J23" s="58" t="s">
         <v>42</v>
       </c>
       <c r="K23" s="9"/>
@@ -2331,32 +2347,32 @@
       <c r="Q23" s="9"/>
     </row>
     <row r="24" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A24" s="62" t="s">
+      <c r="A24" s="100" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="63"/>
-      <c r="C24" s="59" t="s">
+      <c r="B24" s="101"/>
+      <c r="C24" s="95" t="s">
         <v>16</v>
       </c>
       <c r="D24" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="E24" s="100">
+      <c r="E24" s="72">
         <v>600</v>
       </c>
-      <c r="F24" s="101">
+      <c r="F24" s="73">
         <v>600</v>
       </c>
-      <c r="G24" s="100">
+      <c r="G24" s="72">
         <v>600</v>
       </c>
-      <c r="H24" s="101">
+      <c r="H24" s="73">
         <v>600</v>
       </c>
-      <c r="I24" s="100">
+      <c r="I24" s="72">
         <v>600</v>
       </c>
-      <c r="J24" s="74" t="s">
+      <c r="J24" s="55" t="s">
         <v>43</v>
       </c>
       <c r="K24" s="9"/>
@@ -2368,28 +2384,28 @@
       <c r="Q24" s="9"/>
     </row>
     <row r="25" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A25" s="64"/>
-      <c r="B25" s="64"/>
-      <c r="C25" s="59"/>
-      <c r="D25" s="76" t="s">
+      <c r="A25" s="102"/>
+      <c r="B25" s="102"/>
+      <c r="C25" s="95"/>
+      <c r="D25" s="57" t="s">
         <v>48</v>
       </c>
-      <c r="E25" s="100">
+      <c r="E25" s="72">
         <v>100</v>
       </c>
-      <c r="F25" s="101">
+      <c r="F25" s="73">
         <v>100</v>
       </c>
-      <c r="G25" s="100">
+      <c r="G25" s="72">
         <v>100</v>
       </c>
-      <c r="H25" s="101">
+      <c r="H25" s="73">
         <v>100</v>
       </c>
-      <c r="I25" s="100">
+      <c r="I25" s="72">
         <v>100</v>
       </c>
-      <c r="J25" s="74" t="s">
+      <c r="J25" s="55" t="s">
         <v>43</v>
       </c>
       <c r="K25" s="9"/>
@@ -2401,34 +2417,34 @@
       <c r="Q25" s="9"/>
     </row>
     <row r="26" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A26" s="64"/>
-      <c r="B26" s="64"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="76" t="s">
+      <c r="A26" s="102"/>
+      <c r="B26" s="102"/>
+      <c r="C26" s="95"/>
+      <c r="D26" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="E26" s="100">
+      <c r="E26" s="72">
         <v>200</v>
       </c>
-      <c r="F26" s="101">
+      <c r="F26" s="73">
         <v>200</v>
       </c>
-      <c r="G26" s="100">
+      <c r="G26" s="72">
         <v>200</v>
       </c>
-      <c r="H26" s="101">
+      <c r="H26" s="73">
         <v>200</v>
       </c>
-      <c r="I26" s="100">
+      <c r="I26" s="72">
         <v>200</v>
       </c>
-      <c r="J26" s="74" t="s">
+      <c r="J26" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="K26" s="97" t="s">
+      <c r="K26" s="81" t="s">
         <v>74</v>
       </c>
-      <c r="L26" s="98"/>
+      <c r="L26" s="82"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9"/>
       <c r="O26" s="9"/>
@@ -2436,16 +2452,16 @@
       <c r="Q26" s="9"/>
     </row>
     <row r="27" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A27" s="64"/>
-      <c r="B27" s="64"/>
+      <c r="A27" s="102"/>
+      <c r="B27" s="102"/>
       <c r="C27" s="52"/>
       <c r="D27" s="28"/>
-      <c r="E27" s="104"/>
-      <c r="F27" s="105"/>
-      <c r="G27" s="104"/>
-      <c r="H27" s="105"/>
-      <c r="I27" s="104"/>
-      <c r="J27" s="75"/>
+      <c r="E27" s="76"/>
+      <c r="F27" s="77"/>
+      <c r="G27" s="76"/>
+      <c r="H27" s="77"/>
+      <c r="I27" s="76"/>
+      <c r="J27" s="56"/>
       <c r="K27" s="9"/>
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
@@ -2455,30 +2471,30 @@
       <c r="Q27" s="9"/>
     </row>
     <row r="28" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A28" s="64"/>
-      <c r="B28" s="64"/>
-      <c r="C28" s="77" t="s">
+      <c r="A28" s="102"/>
+      <c r="B28" s="102"/>
+      <c r="C28" s="96" t="s">
         <v>2</v>
       </c>
-      <c r="D28" s="76" t="s">
+      <c r="D28" s="57" t="s">
         <v>45</v>
       </c>
-      <c r="E28" s="100">
+      <c r="E28" s="72">
         <v>270</v>
       </c>
-      <c r="F28" s="101">
+      <c r="F28" s="73">
         <v>270</v>
       </c>
-      <c r="G28" s="100">
+      <c r="G28" s="72">
         <v>270</v>
       </c>
-      <c r="H28" s="101">
+      <c r="H28" s="73">
         <v>270</v>
       </c>
-      <c r="I28" s="100">
+      <c r="I28" s="72">
         <v>270</v>
       </c>
-      <c r="J28" s="74" t="s">
+      <c r="J28" s="55" t="s">
         <v>44</v>
       </c>
       <c r="K28" s="9"/>
@@ -2490,28 +2506,28 @@
       <c r="Q28" s="9"/>
     </row>
     <row r="29" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A29" s="64"/>
-      <c r="B29" s="64"/>
-      <c r="C29" s="59"/>
-      <c r="D29" s="76" t="s">
+      <c r="A29" s="102"/>
+      <c r="B29" s="102"/>
+      <c r="C29" s="95"/>
+      <c r="D29" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="100">
+      <c r="E29" s="72">
         <v>57.5</v>
       </c>
-      <c r="F29" s="101">
+      <c r="F29" s="73">
         <v>57.5</v>
       </c>
-      <c r="G29" s="100">
+      <c r="G29" s="72">
         <v>57.5</v>
       </c>
-      <c r="H29" s="101">
+      <c r="H29" s="73">
         <v>57.5</v>
       </c>
-      <c r="I29" s="100">
+      <c r="I29" s="72">
         <v>57.5</v>
       </c>
-      <c r="J29" s="74" t="s">
+      <c r="J29" s="55" t="s">
         <v>49</v>
       </c>
       <c r="K29" s="9"/>
@@ -2523,34 +2539,34 @@
       <c r="Q29" s="9"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A30" s="64"/>
-      <c r="B30" s="64"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="76" t="s">
+      <c r="A30" s="102"/>
+      <c r="B30" s="102"/>
+      <c r="C30" s="95"/>
+      <c r="D30" s="57" t="s">
         <v>70</v>
       </c>
-      <c r="E30" s="100">
+      <c r="E30" s="72">
         <v>145.25</v>
       </c>
-      <c r="F30" s="101">
+      <c r="F30" s="73">
         <v>145.25</v>
       </c>
-      <c r="G30" s="100">
+      <c r="G30" s="72">
         <v>145.25</v>
       </c>
-      <c r="H30" s="101">
+      <c r="H30" s="73">
         <v>145.25</v>
       </c>
-      <c r="I30" s="100">
+      <c r="I30" s="72">
         <v>145.25</v>
       </c>
-      <c r="J30" s="74" t="s">
+      <c r="J30" s="55" t="s">
         <v>71</v>
       </c>
-      <c r="K30" s="97" t="s">
+      <c r="K30" s="81" t="s">
         <v>73</v>
       </c>
-      <c r="L30" s="98"/>
+      <c r="L30" s="82"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9"/>
       <c r="O30" s="9"/>
@@ -2558,16 +2574,16 @@
       <c r="Q30" s="9"/>
     </row>
     <row r="31" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A31" s="64"/>
-      <c r="B31" s="64"/>
+      <c r="A31" s="102"/>
+      <c r="B31" s="102"/>
       <c r="C31" s="52"/>
       <c r="D31" s="28"/>
-      <c r="E31" s="104"/>
-      <c r="F31" s="105"/>
-      <c r="G31" s="104"/>
-      <c r="H31" s="105"/>
-      <c r="I31" s="104"/>
-      <c r="J31" s="75"/>
+      <c r="E31" s="76"/>
+      <c r="F31" s="77"/>
+      <c r="G31" s="76"/>
+      <c r="H31" s="77"/>
+      <c r="I31" s="76"/>
+      <c r="J31" s="56"/>
       <c r="K31" s="9"/>
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
@@ -2577,36 +2593,36 @@
       <c r="Q31" s="9"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A32" s="64"/>
-      <c r="B32" s="64"/>
-      <c r="C32" s="78" t="s">
+      <c r="A32" s="102"/>
+      <c r="B32" s="102"/>
+      <c r="C32" s="98" t="s">
         <v>47</v>
       </c>
-      <c r="D32" s="76" t="s">
+      <c r="D32" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="E32" s="100">
+      <c r="E32" s="72">
         <v>3000</v>
       </c>
-      <c r="F32" s="101">
+      <c r="F32" s="73">
         <v>3000</v>
       </c>
-      <c r="G32" s="100">
+      <c r="G32" s="72">
         <v>3000</v>
       </c>
-      <c r="H32" s="101">
+      <c r="H32" s="73">
         <v>3000</v>
       </c>
-      <c r="I32" s="100">
+      <c r="I32" s="72">
         <v>3000</v>
       </c>
-      <c r="J32" s="74" t="s">
+      <c r="J32" s="55" t="s">
         <v>50</v>
       </c>
-      <c r="K32" s="97" t="s">
+      <c r="K32" s="81" t="s">
         <v>75</v>
       </c>
-      <c r="L32" s="98"/>
+      <c r="L32" s="82"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9"/>
       <c r="O32" s="9"/>
@@ -2614,34 +2630,34 @@
       <c r="Q32" s="9"/>
     </row>
     <row r="33" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A33" s="64"/>
-      <c r="B33" s="64"/>
-      <c r="C33" s="60"/>
-      <c r="D33" s="76" t="s">
+      <c r="A33" s="102"/>
+      <c r="B33" s="102"/>
+      <c r="C33" s="99"/>
+      <c r="D33" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="100">
+      <c r="E33" s="72">
         <v>500</v>
       </c>
-      <c r="F33" s="101">
+      <c r="F33" s="73">
         <v>500</v>
       </c>
-      <c r="G33" s="100">
+      <c r="G33" s="72">
         <v>500</v>
       </c>
-      <c r="H33" s="101">
+      <c r="H33" s="73">
         <v>500</v>
       </c>
-      <c r="I33" s="100">
+      <c r="I33" s="72">
         <v>500</v>
       </c>
-      <c r="J33" s="74" t="s">
+      <c r="J33" s="55" t="s">
         <v>50</v>
       </c>
-      <c r="K33" s="97" t="s">
+      <c r="K33" s="81" t="s">
         <v>76</v>
       </c>
-      <c r="L33" s="98"/>
+      <c r="L33" s="82"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9"/>
       <c r="O33" s="9"/>
@@ -2649,16 +2665,16 @@
       <c r="Q33" s="9"/>
     </row>
     <row r="34" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A34" s="64"/>
-      <c r="B34" s="64"/>
+      <c r="A34" s="102"/>
+      <c r="B34" s="102"/>
       <c r="C34" s="52"/>
       <c r="D34" s="28"/>
-      <c r="E34" s="104"/>
-      <c r="F34" s="105"/>
-      <c r="G34" s="104"/>
-      <c r="H34" s="105"/>
-      <c r="I34" s="104"/>
-      <c r="J34" s="75"/>
+      <c r="E34" s="76"/>
+      <c r="F34" s="77"/>
+      <c r="G34" s="76"/>
+      <c r="H34" s="77"/>
+      <c r="I34" s="76"/>
+      <c r="J34" s="56"/>
       <c r="K34" s="9"/>
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
@@ -2668,16 +2684,16 @@
       <c r="Q34" s="9"/>
     </row>
     <row r="35" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A35" s="64"/>
-      <c r="B35" s="64"/>
+      <c r="A35" s="102"/>
+      <c r="B35" s="102"/>
       <c r="C35" s="52"/>
       <c r="D35" s="28"/>
-      <c r="E35" s="104"/>
-      <c r="F35" s="105"/>
-      <c r="G35" s="104"/>
-      <c r="H35" s="105"/>
-      <c r="I35" s="104"/>
-      <c r="J35" s="75"/>
+      <c r="E35" s="76"/>
+      <c r="F35" s="77"/>
+      <c r="G35" s="76"/>
+      <c r="H35" s="77"/>
+      <c r="I35" s="76"/>
+      <c r="J35" s="56"/>
       <c r="K35" s="9"/>
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
@@ -2687,30 +2703,30 @@
       <c r="Q35" s="9"/>
     </row>
     <row r="36" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A36" s="64"/>
-      <c r="B36" s="64"/>
+      <c r="A36" s="102"/>
+      <c r="B36" s="102"/>
       <c r="C36" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="D36" s="76" t="s">
+      <c r="D36" s="57" t="s">
         <v>56</v>
       </c>
-      <c r="E36" s="100">
+      <c r="E36" s="72">
         <v>840</v>
       </c>
-      <c r="F36" s="101">
+      <c r="F36" s="73">
         <v>840</v>
       </c>
-      <c r="G36" s="100">
+      <c r="G36" s="72">
         <v>840</v>
       </c>
-      <c r="H36" s="101">
+      <c r="H36" s="73">
         <v>840</v>
       </c>
-      <c r="I36" s="100">
+      <c r="I36" s="72">
         <v>840</v>
       </c>
-      <c r="J36" s="74" t="s">
+      <c r="J36" s="55" t="s">
         <v>43</v>
       </c>
       <c r="K36" s="9"/>
@@ -2722,8 +2738,8 @@
       <c r="Q36" s="9"/>
     </row>
     <row r="37" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A37" s="64"/>
-      <c r="B37" s="64"/>
+      <c r="A37" s="102"/>
+      <c r="B37" s="102"/>
       <c r="C37" s="28"/>
       <c r="D37" s="28"/>
       <c r="E37" s="26"/>
@@ -2741,8 +2757,8 @@
       <c r="Q37" s="9"/>
     </row>
     <row r="38" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A38" s="64"/>
-      <c r="B38" s="64"/>
+      <c r="A38" s="102"/>
+      <c r="B38" s="102"/>
       <c r="C38" s="33" t="s">
         <v>20</v>
       </c>
@@ -2777,8 +2793,8 @@
       <c r="Q38" s="9"/>
     </row>
     <row r="39" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A39" s="64"/>
-      <c r="B39" s="64"/>
+      <c r="A39" s="102"/>
+      <c r="B39" s="102"/>
       <c r="C39" s="28"/>
       <c r="D39" s="28"/>
       <c r="E39" s="26"/>
@@ -2796,8 +2812,8 @@
       <c r="Q39" s="9"/>
     </row>
     <row r="40" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A40" s="64"/>
-      <c r="B40" s="64"/>
+      <c r="A40" s="102"/>
+      <c r="B40" s="102"/>
       <c r="C40" s="33" t="s">
         <v>26</v>
       </c>
@@ -2851,29 +2867,29 @@
       <c r="Q41" s="9"/>
     </row>
     <row r="42" spans="1:17">
-      <c r="A42" s="61" t="s">
+      <c r="A42" s="97" t="s">
         <v>32</v>
       </c>
-      <c r="B42" s="61"/>
-      <c r="C42" s="59" t="s">
+      <c r="B42" s="97"/>
+      <c r="C42" s="95" t="s">
         <v>16</v>
       </c>
       <c r="D42" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E42" s="100">
+      <c r="E42" s="72">
         <v>90</v>
       </c>
-      <c r="F42" s="101">
+      <c r="F42" s="73">
         <v>84</v>
       </c>
-      <c r="G42" s="102" t="s">
+      <c r="G42" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H42" s="103" t="s">
+      <c r="H42" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I42" s="102" t="s">
+      <c r="I42" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J42" s="13"/>
@@ -2886,25 +2902,25 @@
       <c r="Q42" s="9"/>
     </row>
     <row r="43" spans="1:17">
-      <c r="A43" s="61"/>
-      <c r="B43" s="61"/>
-      <c r="C43" s="59"/>
+      <c r="A43" s="97"/>
+      <c r="B43" s="97"/>
+      <c r="C43" s="95"/>
       <c r="D43" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="E43" s="100">
+      <c r="E43" s="72">
         <v>20</v>
       </c>
-      <c r="F43" s="101">
+      <c r="F43" s="73">
         <v>14.35</v>
       </c>
-      <c r="G43" s="102" t="s">
+      <c r="G43" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H43" s="103" t="s">
+      <c r="H43" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I43" s="102" t="s">
+      <c r="I43" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J43" s="13"/>
@@ -2917,25 +2933,25 @@
       <c r="Q43" s="9"/>
     </row>
     <row r="44" spans="1:17">
-      <c r="A44" s="61"/>
-      <c r="B44" s="61"/>
-      <c r="C44" s="59"/>
+      <c r="A44" s="97"/>
+      <c r="B44" s="97"/>
+      <c r="C44" s="95"/>
       <c r="D44" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="E44" s="100">
+      <c r="E44" s="72">
         <v>19.899999999999999</v>
       </c>
-      <c r="F44" s="101">
+      <c r="F44" s="73">
         <v>15.5</v>
       </c>
-      <c r="G44" s="102" t="s">
+      <c r="G44" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H44" s="103" t="s">
+      <c r="H44" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I44" s="102" t="s">
+      <c r="I44" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J44" s="13"/>
@@ -2948,25 +2964,25 @@
       <c r="Q44" s="9"/>
     </row>
     <row r="45" spans="1:17">
-      <c r="A45" s="61"/>
-      <c r="B45" s="61"/>
-      <c r="C45" s="59"/>
+      <c r="A45" s="97"/>
+      <c r="B45" s="97"/>
+      <c r="C45" s="95"/>
       <c r="D45" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="E45" s="100">
+      <c r="E45" s="72">
         <v>25</v>
       </c>
-      <c r="F45" s="101">
+      <c r="F45" s="73">
         <v>20</v>
       </c>
-      <c r="G45" s="102" t="s">
+      <c r="G45" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H45" s="103" t="s">
+      <c r="H45" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I45" s="102" t="s">
+      <c r="I45" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J45" s="13"/>
@@ -2979,25 +2995,25 @@
       <c r="Q45" s="9"/>
     </row>
     <row r="46" spans="1:17">
-      <c r="A46" s="61"/>
-      <c r="B46" s="61"/>
-      <c r="C46" s="59"/>
+      <c r="A46" s="97"/>
+      <c r="B46" s="97"/>
+      <c r="C46" s="95"/>
       <c r="D46" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="E46" s="100">
+      <c r="E46" s="72">
         <v>120</v>
       </c>
-      <c r="F46" s="101">
+      <c r="F46" s="73">
         <v>79</v>
       </c>
-      <c r="G46" s="102" t="s">
+      <c r="G46" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H46" s="103" t="s">
+      <c r="H46" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I46" s="102" t="s">
+      <c r="I46" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J46" s="13"/>
@@ -3010,19 +3026,19 @@
       <c r="Q46" s="9"/>
     </row>
     <row r="47" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A47" s="61"/>
-      <c r="B47" s="61"/>
+      <c r="A47" s="97"/>
+      <c r="B47" s="97"/>
       <c r="C47" s="52"/>
       <c r="D47" s="28"/>
-      <c r="E47" s="106"/>
-      <c r="F47" s="107"/>
-      <c r="G47" s="102" t="s">
+      <c r="E47" s="78"/>
+      <c r="F47" s="79"/>
+      <c r="G47" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H47" s="103" t="s">
+      <c r="H47" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I47" s="102" t="s">
+      <c r="I47" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J47" s="13"/>
@@ -3035,27 +3051,27 @@
       <c r="Q47" s="9"/>
     </row>
     <row r="48" spans="1:17">
-      <c r="A48" s="61"/>
-      <c r="B48" s="61"/>
-      <c r="C48" s="77" t="s">
+      <c r="A48" s="97"/>
+      <c r="B48" s="97"/>
+      <c r="C48" s="96" t="s">
         <v>51</v>
       </c>
-      <c r="D48" s="76" t="s">
+      <c r="D48" s="57" t="s">
         <v>45</v>
       </c>
-      <c r="E48" s="100">
+      <c r="E48" s="72">
         <v>35</v>
       </c>
-      <c r="F48" s="101">
+      <c r="F48" s="73">
         <v>10</v>
       </c>
-      <c r="G48" s="102" t="s">
+      <c r="G48" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H48" s="103" t="s">
+      <c r="H48" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I48" s="102" t="s">
+      <c r="I48" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J48" s="13"/>
@@ -3068,25 +3084,25 @@
       <c r="Q48" s="9"/>
     </row>
     <row r="49" spans="1:17">
-      <c r="A49" s="61"/>
-      <c r="B49" s="61"/>
-      <c r="C49" s="59"/>
-      <c r="D49" s="76" t="s">
+      <c r="A49" s="97"/>
+      <c r="B49" s="97"/>
+      <c r="C49" s="95"/>
+      <c r="D49" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="100">
+      <c r="E49" s="72">
         <v>16</v>
       </c>
-      <c r="F49" s="101">
+      <c r="F49" s="73">
         <v>27</v>
       </c>
-      <c r="G49" s="102" t="s">
+      <c r="G49" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H49" s="103" t="s">
+      <c r="H49" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I49" s="102" t="s">
+      <c r="I49" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J49" s="13"/>
@@ -3099,8 +3115,8 @@
       <c r="Q49" s="9"/>
     </row>
     <row r="50" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A50" s="61"/>
-      <c r="B50" s="61"/>
+      <c r="A50" s="97"/>
+      <c r="B50" s="97"/>
       <c r="C50" s="53"/>
       <c r="D50" s="28"/>
       <c r="E50" s="36"/>
@@ -3118,8 +3134,8 @@
       <c r="Q50" s="9"/>
     </row>
     <row r="51" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A51" s="61"/>
-      <c r="B51" s="61"/>
+      <c r="A51" s="97"/>
+      <c r="B51" s="97"/>
       <c r="C51" s="38"/>
       <c r="D51" s="28"/>
       <c r="E51" s="26"/>
@@ -3137,8 +3153,8 @@
       <c r="Q51" s="9"/>
     </row>
     <row r="52" spans="1:17">
-      <c r="A52" s="61"/>
-      <c r="B52" s="61"/>
+      <c r="A52" s="97"/>
+      <c r="B52" s="97"/>
       <c r="C52" s="39" t="s">
         <v>21</v>
       </c>
@@ -3173,8 +3189,8 @@
       <c r="Q52" s="9"/>
     </row>
     <row r="53" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A53" s="61"/>
-      <c r="B53" s="61"/>
+      <c r="A53" s="97"/>
+      <c r="B53" s="97"/>
       <c r="C53" s="28"/>
       <c r="D53" s="28"/>
       <c r="E53" s="26"/>
@@ -3192,8 +3208,8 @@
       <c r="Q53" s="9"/>
     </row>
     <row r="54" spans="1:17">
-      <c r="A54" s="61"/>
-      <c r="B54" s="61"/>
+      <c r="A54" s="97"/>
+      <c r="B54" s="97"/>
       <c r="C54" s="33" t="s">
         <v>26</v>
       </c>
@@ -3247,29 +3263,29 @@
       <c r="Q55" s="9"/>
     </row>
     <row r="56" spans="1:17">
-      <c r="A56" s="61" t="s">
+      <c r="A56" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="B56" s="61"/>
-      <c r="C56" s="77" t="s">
+      <c r="B56" s="97"/>
+      <c r="C56" s="96" t="s">
         <v>52</v>
       </c>
-      <c r="D56" s="76" t="s">
+      <c r="D56" s="57" t="s">
         <v>53</v>
       </c>
-      <c r="E56" s="100">
+      <c r="E56" s="72">
         <v>320</v>
       </c>
-      <c r="F56" s="101">
+      <c r="F56" s="73">
         <v>210</v>
       </c>
-      <c r="G56" s="102" t="s">
+      <c r="G56" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H56" s="103" t="s">
+      <c r="H56" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I56" s="102" t="s">
+      <c r="I56" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J56" s="13"/>
@@ -3282,25 +3298,25 @@
       <c r="Q56" s="9"/>
     </row>
     <row r="57" spans="1:17">
-      <c r="A57" s="61"/>
-      <c r="B57" s="61"/>
-      <c r="C57" s="59"/>
-      <c r="D57" s="76" t="s">
+      <c r="A57" s="97"/>
+      <c r="B57" s="97"/>
+      <c r="C57" s="95"/>
+      <c r="D57" s="57" t="s">
         <v>54</v>
       </c>
-      <c r="E57" s="100">
+      <c r="E57" s="72">
         <v>125</v>
       </c>
-      <c r="F57" s="101">
+      <c r="F57" s="73">
         <v>45</v>
       </c>
-      <c r="G57" s="102" t="s">
+      <c r="G57" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H57" s="103" t="s">
+      <c r="H57" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I57" s="102" t="s">
+      <c r="I57" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J57" s="13"/>
@@ -3313,25 +3329,25 @@
       <c r="Q57" s="9"/>
     </row>
     <row r="58" spans="1:17">
-      <c r="A58" s="61"/>
-      <c r="B58" s="61"/>
-      <c r="C58" s="59"/>
-      <c r="D58" s="76" t="s">
+      <c r="A58" s="97"/>
+      <c r="B58" s="97"/>
+      <c r="C58" s="95"/>
+      <c r="D58" s="57" t="s">
         <v>55</v>
       </c>
-      <c r="E58" s="100">
+      <c r="E58" s="72">
         <v>100</v>
       </c>
-      <c r="F58" s="101">
+      <c r="F58" s="73">
         <v>30</v>
       </c>
-      <c r="G58" s="102" t="s">
+      <c r="G58" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H58" s="103" t="s">
+      <c r="H58" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I58" s="102" t="s">
+      <c r="I58" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J58" s="13"/>
@@ -3344,8 +3360,8 @@
       <c r="Q58" s="9"/>
     </row>
     <row r="59" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A59" s="61"/>
-      <c r="B59" s="61"/>
+      <c r="A59" s="97"/>
+      <c r="B59" s="97"/>
       <c r="C59" s="53"/>
       <c r="D59" s="28"/>
       <c r="E59" s="36"/>
@@ -3363,8 +3379,8 @@
       <c r="Q59" s="9"/>
     </row>
     <row r="60" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A60" s="61"/>
-      <c r="B60" s="61"/>
+      <c r="A60" s="97"/>
+      <c r="B60" s="97"/>
       <c r="C60" s="37"/>
       <c r="D60" s="28"/>
       <c r="E60" s="36"/>
@@ -3382,8 +3398,8 @@
       <c r="Q60" s="9"/>
     </row>
     <row r="61" spans="1:17">
-      <c r="A61" s="61"/>
-      <c r="B61" s="61"/>
+      <c r="A61" s="97"/>
+      <c r="B61" s="97"/>
       <c r="C61" s="33" t="s">
         <v>22</v>
       </c>
@@ -3418,8 +3434,8 @@
       <c r="Q61" s="9"/>
     </row>
     <row r="62" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A62" s="61"/>
-      <c r="B62" s="61"/>
+      <c r="A62" s="97"/>
+      <c r="B62" s="97"/>
       <c r="C62" s="28"/>
       <c r="D62" s="28"/>
       <c r="E62" s="26"/>
@@ -3437,8 +3453,8 @@
       <c r="Q62" s="9"/>
     </row>
     <row r="63" spans="1:17">
-      <c r="A63" s="61"/>
-      <c r="B63" s="61"/>
+      <c r="A63" s="97"/>
+      <c r="B63" s="97"/>
       <c r="C63" s="33" t="s">
         <v>26</v>
       </c>
@@ -3492,29 +3508,29 @@
       <c r="Q64" s="9"/>
     </row>
     <row r="65" spans="1:17">
-      <c r="A65" s="61" t="s">
+      <c r="A65" s="97" t="s">
         <v>34</v>
       </c>
-      <c r="B65" s="61"/>
-      <c r="C65" s="59" t="s">
+      <c r="B65" s="97"/>
+      <c r="C65" s="95" t="s">
         <v>38</v>
       </c>
       <c r="D65" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="E65" s="100">
+      <c r="E65" s="72">
         <v>142</v>
       </c>
-      <c r="F65" s="103">
+      <c r="F65" s="75">
         <v>0</v>
       </c>
-      <c r="G65" s="102" t="s">
+      <c r="G65" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H65" s="103" t="s">
+      <c r="H65" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I65" s="102" t="s">
+      <c r="I65" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J65" s="13"/>
@@ -3527,25 +3543,25 @@
       <c r="Q65" s="9"/>
     </row>
     <row r="66" spans="1:17">
-      <c r="A66" s="61"/>
-      <c r="B66" s="61"/>
-      <c r="C66" s="59"/>
-      <c r="D66" s="76" t="s">
+      <c r="A66" s="97"/>
+      <c r="B66" s="97"/>
+      <c r="C66" s="95"/>
+      <c r="D66" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="E66" s="100">
+      <c r="E66" s="72">
         <v>40</v>
       </c>
-      <c r="F66" s="103">
+      <c r="F66" s="75">
         <v>0</v>
       </c>
-      <c r="G66" s="102" t="s">
+      <c r="G66" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H66" s="103" t="s">
+      <c r="H66" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I66" s="102" t="s">
+      <c r="I66" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J66" s="13"/>
@@ -3558,25 +3574,25 @@
       <c r="Q66" s="9"/>
     </row>
     <row r="67" spans="1:17">
-      <c r="A67" s="61"/>
-      <c r="B67" s="61"/>
-      <c r="C67" s="59"/>
+      <c r="A67" s="97"/>
+      <c r="B67" s="97"/>
+      <c r="C67" s="95"/>
       <c r="D67" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="E67" s="100">
+      <c r="E67" s="72">
         <v>83.84</v>
       </c>
-      <c r="F67" s="103">
+      <c r="F67" s="75">
         <v>0</v>
       </c>
-      <c r="G67" s="102" t="s">
+      <c r="G67" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H67" s="103" t="s">
+      <c r="H67" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I67" s="102" t="s">
+      <c r="I67" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J67" s="13"/>
@@ -3589,25 +3605,25 @@
       <c r="Q67" s="9"/>
     </row>
     <row r="68" spans="1:17">
-      <c r="A68" s="61"/>
-      <c r="B68" s="61"/>
-      <c r="C68" s="59"/>
-      <c r="D68" s="76" t="s">
+      <c r="A68" s="97"/>
+      <c r="B68" s="97"/>
+      <c r="C68" s="95"/>
+      <c r="D68" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="E68" s="100">
+      <c r="E68" s="72">
         <v>350</v>
       </c>
-      <c r="F68" s="101">
+      <c r="F68" s="73">
         <v>500</v>
       </c>
-      <c r="G68" s="102" t="s">
+      <c r="G68" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H68" s="103" t="s">
+      <c r="H68" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I68" s="102" t="s">
+      <c r="I68" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J68" s="13"/>
@@ -3620,19 +3636,19 @@
       <c r="Q68" s="9"/>
     </row>
     <row r="69" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A69" s="61"/>
-      <c r="B69" s="61"/>
+      <c r="A69" s="97"/>
+      <c r="B69" s="97"/>
       <c r="C69" s="53"/>
       <c r="D69" s="28"/>
-      <c r="E69" s="106"/>
-      <c r="F69" s="107"/>
-      <c r="G69" s="102" t="s">
+      <c r="E69" s="78"/>
+      <c r="F69" s="79"/>
+      <c r="G69" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H69" s="103" t="s">
+      <c r="H69" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I69" s="102" t="s">
+      <c r="I69" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J69" s="13"/>
@@ -3645,27 +3661,27 @@
       <c r="Q69" s="9"/>
     </row>
     <row r="70" spans="1:17">
-      <c r="A70" s="61"/>
-      <c r="B70" s="61"/>
-      <c r="C70" s="80" t="s">
+      <c r="A70" s="97"/>
+      <c r="B70" s="97"/>
+      <c r="C70" s="59" t="s">
         <v>58</v>
       </c>
-      <c r="D70" s="76" t="s">
+      <c r="D70" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="E70" s="100">
+      <c r="E70" s="72">
         <v>774.16</v>
       </c>
-      <c r="F70" s="101">
+      <c r="F70" s="73">
         <v>134.1</v>
       </c>
-      <c r="G70" s="102" t="s">
+      <c r="G70" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="H70" s="103" t="s">
+      <c r="H70" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="I70" s="102" t="s">
+      <c r="I70" s="74" t="s">
         <v>72</v>
       </c>
       <c r="J70" s="13"/>
@@ -3678,8 +3694,8 @@
       <c r="Q70" s="9"/>
     </row>
     <row r="71" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A71" s="61"/>
-      <c r="B71" s="61"/>
+      <c r="A71" s="97"/>
+      <c r="B71" s="97"/>
       <c r="C71" s="38"/>
       <c r="D71" s="28"/>
       <c r="E71" s="26"/>
@@ -3697,8 +3713,8 @@
       <c r="Q71" s="9"/>
     </row>
     <row r="72" spans="1:17">
-      <c r="A72" s="61"/>
-      <c r="B72" s="61"/>
+      <c r="A72" s="97"/>
+      <c r="B72" s="97"/>
       <c r="C72" s="33" t="s">
         <v>28</v>
       </c>
@@ -3733,8 +3749,8 @@
       <c r="Q72" s="9"/>
     </row>
     <row r="73" spans="1:17" ht="3.75" customHeight="1">
-      <c r="A73" s="61"/>
-      <c r="B73" s="61"/>
+      <c r="A73" s="97"/>
+      <c r="B73" s="97"/>
       <c r="C73" s="28"/>
       <c r="D73" s="28"/>
       <c r="E73" s="26"/>
@@ -3752,8 +3768,8 @@
       <c r="Q73" s="9"/>
     </row>
     <row r="74" spans="1:17">
-      <c r="A74" s="61"/>
-      <c r="B74" s="61"/>
+      <c r="A74" s="97"/>
+      <c r="B74" s="97"/>
       <c r="C74" s="33" t="s">
         <v>26</v>
       </c>
@@ -3807,31 +3823,31 @@
       <c r="Q75" s="9"/>
     </row>
     <row r="76" spans="1:17">
-      <c r="A76" s="91" t="s">
+      <c r="A76" s="85" t="s">
         <v>61</v>
       </c>
-      <c r="B76" s="65"/>
-      <c r="C76" s="66"/>
+      <c r="B76" s="86"/>
+      <c r="C76" s="87"/>
       <c r="D76" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E76" s="108">
+      <c r="E76" s="80">
         <f>E9</f>
         <v>7973.65</v>
       </c>
-      <c r="F76" s="108">
+      <c r="F76" s="80">
         <f>F9</f>
         <v>4026.35</v>
       </c>
-      <c r="G76" s="108">
+      <c r="G76" s="80">
         <f>G9</f>
         <v>0</v>
       </c>
-      <c r="H76" s="108">
+      <c r="H76" s="80">
         <f>H9</f>
         <v>0</v>
       </c>
-      <c r="I76" s="108">
+      <c r="I76" s="80">
         <f>I9</f>
         <v>0</v>
       </c>
@@ -3845,29 +3861,29 @@
       <c r="Q76" s="9"/>
     </row>
     <row r="77" spans="1:17">
-      <c r="A77" s="67"/>
-      <c r="B77" s="68"/>
-      <c r="C77" s="69"/>
+      <c r="A77" s="88"/>
+      <c r="B77" s="89"/>
+      <c r="C77" s="90"/>
       <c r="D77" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="E77" s="108">
+      <c r="E77" s="80">
         <f>E38</f>
         <v>5712.75</v>
       </c>
-      <c r="F77" s="108">
+      <c r="F77" s="80">
         <f>F38</f>
         <v>5712.75</v>
       </c>
-      <c r="G77" s="108">
+      <c r="G77" s="80">
         <f>G38</f>
         <v>5712.75</v>
       </c>
-      <c r="H77" s="108">
+      <c r="H77" s="80">
         <f>H38</f>
         <v>5712.75</v>
       </c>
-      <c r="I77" s="108">
+      <c r="I77" s="80">
         <f>I38</f>
         <v>5712.75</v>
       </c>
@@ -3881,29 +3897,29 @@
       <c r="Q77" s="9"/>
     </row>
     <row r="78" spans="1:17">
-      <c r="A78" s="67"/>
-      <c r="B78" s="68"/>
-      <c r="C78" s="69"/>
+      <c r="A78" s="88"/>
+      <c r="B78" s="89"/>
+      <c r="C78" s="90"/>
       <c r="D78" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="E78" s="108">
+      <c r="E78" s="80">
         <f>E52</f>
         <v>325.89999999999998</v>
       </c>
-      <c r="F78" s="108">
+      <c r="F78" s="80">
         <f>F52</f>
         <v>249.85</v>
       </c>
-      <c r="G78" s="108">
+      <c r="G78" s="80">
         <f>G52</f>
         <v>0</v>
       </c>
-      <c r="H78" s="108">
+      <c r="H78" s="80">
         <f>H52</f>
         <v>0</v>
       </c>
-      <c r="I78" s="108">
+      <c r="I78" s="80">
         <f>I52</f>
         <v>0</v>
       </c>
@@ -3917,29 +3933,29 @@
       <c r="Q78" s="9"/>
     </row>
     <row r="79" spans="1:17">
-      <c r="A79" s="67"/>
-      <c r="B79" s="68"/>
-      <c r="C79" s="69"/>
+      <c r="A79" s="88"/>
+      <c r="B79" s="89"/>
+      <c r="C79" s="90"/>
       <c r="D79" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="E79" s="108">
+      <c r="E79" s="80">
         <f>E61</f>
         <v>545</v>
       </c>
-      <c r="F79" s="108">
+      <c r="F79" s="80">
         <f>F61</f>
         <v>285</v>
       </c>
-      <c r="G79" s="108">
+      <c r="G79" s="80">
         <f>G61</f>
         <v>0</v>
       </c>
-      <c r="H79" s="108">
+      <c r="H79" s="80">
         <f>H61</f>
         <v>0</v>
       </c>
-      <c r="I79" s="108">
+      <c r="I79" s="80">
         <f>I61</f>
         <v>0</v>
       </c>
@@ -3953,29 +3969,29 @@
       <c r="Q79" s="9"/>
     </row>
     <row r="80" spans="1:17">
-      <c r="A80" s="67"/>
-      <c r="B80" s="68"/>
-      <c r="C80" s="69"/>
+      <c r="A80" s="88"/>
+      <c r="B80" s="89"/>
+      <c r="C80" s="90"/>
       <c r="D80" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="E80" s="108">
+      <c r="E80" s="80">
         <f>E72</f>
         <v>1390</v>
       </c>
-      <c r="F80" s="108">
+      <c r="F80" s="80">
         <f>F72</f>
         <v>634.1</v>
       </c>
-      <c r="G80" s="108">
+      <c r="G80" s="80">
         <f>G72</f>
         <v>0</v>
       </c>
-      <c r="H80" s="108">
+      <c r="H80" s="80">
         <f>H72</f>
         <v>0</v>
       </c>
-      <c r="I80" s="108">
+      <c r="I80" s="80">
         <f>I72</f>
         <v>0</v>
       </c>
@@ -3989,10 +4005,10 @@
       <c r="Q80" s="9"/>
     </row>
     <row r="81" spans="1:24">
-      <c r="A81" s="70"/>
-      <c r="B81" s="71"/>
-      <c r="C81" s="72"/>
-      <c r="D81" s="99" t="s">
+      <c r="A81" s="91"/>
+      <c r="B81" s="92"/>
+      <c r="C81" s="93"/>
+      <c r="D81" s="71" t="s">
         <v>14</v>
       </c>
       <c r="E81" s="43">
@@ -4028,22 +4044,22 @@
       <c r="A82" s="13"/>
       <c r="B82" s="13"/>
       <c r="C82" s="13"/>
-      <c r="D82" s="95" t="s">
+      <c r="D82" s="69" t="s">
         <v>67</v>
       </c>
-      <c r="E82" s="96" t="s">
+      <c r="E82" s="70" t="s">
         <v>66</v>
       </c>
-      <c r="F82" s="96" t="s">
+      <c r="F82" s="70" t="s">
         <v>69</v>
       </c>
-      <c r="G82" s="96" t="s">
+      <c r="G82" s="70" t="s">
         <v>68</v>
       </c>
-      <c r="H82" s="96" t="s">
+      <c r="H82" s="70" t="s">
         <v>68</v>
       </c>
-      <c r="I82" s="96" t="s">
+      <c r="I82" s="70" t="s">
         <v>68</v>
       </c>
       <c r="J82" s="14"/>
@@ -7600,11 +7616,10 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="A10:C12"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:C9"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A5:D5"/>
     <mergeCell ref="A76:C81"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="C24:C26"/>
@@ -7618,13 +7633,14 @@
     <mergeCell ref="A56:B63"/>
     <mergeCell ref="C48:C49"/>
     <mergeCell ref="A24:B40"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="A10:C12"/>
     <mergeCell ref="A16:C20"/>
     <mergeCell ref="A13:C15"/>
     <mergeCell ref="A21:C22"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A6:C9"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A5:D5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="E81:I81">
@@ -7632,9 +7648,12 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="A5" r:id="rId1" xr:uid="{D2442760-1FDE-48C5-A0D0-C2FA5FEB3160}"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.43" right="0.44" top="0.27" bottom="0.23" header="0.18" footer="0.15"/>
-  <pageSetup paperSize="9" scale="45" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="45" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <headerFooter alignWithMargins="0"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="54" max="16383" man="1"/>
@@ -7642,6 +7661,6 @@
   <ignoredErrors>
     <ignoredError sqref="E40:I40 E54:I54 E63:I63 E74:I74" evalError="1"/>
   </ignoredErrors>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>